<commit_message>
Official experiment including paramgen time and proof verification, db commitment time
</commit_message>
<xml_diff>
--- a/src/zkp-sparql/report/experiment_official_results.xlsx
+++ b/src/zkp-sparql/report/experiment_official_results.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uninsubria365-my.sharepoint.com/personal/qnguyenthanh_studenti_uninsubria_it/Documents/Documents/shinPhD/Experiment-logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="335" documentId="11_66C972AFD3F0D14CB3992311595ED87656CD925F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F05C68E-9430-4A52-AAB7-844691DDAE7E}"/>
+  <xr:revisionPtr revIDLastSave="430" documentId="11_66C972AFD3F0D14CB3992311595ED87656CD925F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{120848EB-5960-494F-9054-3F1E195AC49E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
     <sheet name="25pct" sheetId="2" r:id="rId2"/>
     <sheet name="50pct" sheetId="3" r:id="rId3"/>
     <sheet name="100pct" sheetId="4" r:id="rId4"/>
-    <sheet name="swdf" sheetId="5" r:id="rId5"/>
-    <sheet name="drugbank" sheetId="6" r:id="rId6"/>
-    <sheet name="bsbm" sheetId="7" r:id="rId7"/>
-    <sheet name="bsbm_compared" sheetId="8" r:id="rId8"/>
-    <sheet name="swdf_single_gate" sheetId="9" r:id="rId9"/>
+    <sheet name="param_gen" sheetId="10" r:id="rId5"/>
+    <sheet name="swdf" sheetId="5" r:id="rId6"/>
+    <sheet name="drugbank" sheetId="6" r:id="rId7"/>
+    <sheet name="bsbm" sheetId="7" r:id="rId8"/>
+    <sheet name="bsbm_compared" sheetId="8" r:id="rId9"/>
+    <sheet name="swdf_single_gate" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="50">
   <si>
     <t>Dataset</t>
   </si>
@@ -178,6 +179,18 @@
   <si>
     <t>Slice</t>
   </si>
+  <si>
+    <t>Proving Time</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>Time (s)</t>
+  </si>
+  <si>
+    <t>DB Commitment Time</t>
+  </si>
 </sst>
 </file>
 
@@ -249,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -259,6 +272,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1819,6 +1835,93 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D448E8-895B-453C-BC61-2624AF8420AB}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2">
+        <v>6.3574999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3">
+        <v>94.953100000000006</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4">
+        <v>29.642399999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5">
+        <v>3.3828</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6">
+        <v>1.6611</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7">
+        <v>43.620800000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8">
+        <v>0.41070000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9">
+        <v>0.52849999999999997</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{575985B6-708C-4265-84DE-2A24D7DEAE49}">
   <dimension ref="A1:H16"/>
@@ -3101,8 +3204,58 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FE8BBFA-8401-459C-B898-51C14CA5BDAE}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>1619</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>20</v>
+      </c>
+      <c r="B5">
+        <v>3319</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{178D22CC-A02D-4C62-851D-6FB9CB59C264}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -3111,11 +3264,13 @@
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -3138,19 +3293,25 @@
         <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M1" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>25</v>
       </c>
@@ -3176,17 +3337,23 @@
         <v>8.0802514553070068</v>
       </c>
       <c r="I2">
-        <f>K2/1024</f>
+        <v>158</v>
+      </c>
+      <c r="J2">
+        <f>L2/1024</f>
         <v>2.318623046875</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>6.9</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>2374.27</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>2.6659999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>25</v>
       </c>
@@ -3212,17 +3379,23 @@
         <v>14.14151310920715</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I16" si="0">K3/1024</f>
+        <v>159</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J16" si="0">L3/1024</f>
         <v>2.4676660156249999</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>6.9</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>2526.89</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M3">
+        <v>1.2450000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>25</v>
       </c>
@@ -3248,17 +3421,23 @@
         <v>15.14360785484314</v>
       </c>
       <c r="I4">
+        <v>161</v>
+      </c>
+      <c r="J4">
         <f t="shared" si="0"/>
         <v>2.5052441406249999</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>6.8</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>2565.37</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M4">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>25</v>
       </c>
@@ -3284,17 +3463,23 @@
         <v>6.4740762710571289</v>
       </c>
       <c r="I5">
+        <v>156</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="0"/>
         <v>2.3704199218749999</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>6.9</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>2427.31</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M5">
+        <v>0.76100000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>25</v>
       </c>
@@ -3320,17 +3505,23 @@
         <v>52.294199705123901</v>
       </c>
       <c r="I6">
+        <v>173</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="0"/>
         <v>2.6463378906249999</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>7</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>2709.85</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M6">
+        <v>4.5949999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>50</v>
       </c>
@@ -3356,17 +3547,23 @@
         <v>19.47108888626099</v>
       </c>
       <c r="I7">
+        <v>295</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="0"/>
         <v>4.9627734375000001</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>15</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>5081.88</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M7">
+        <v>3.258</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>50</v>
       </c>
@@ -3392,17 +3589,23 @@
         <v>27.646983623504639</v>
       </c>
       <c r="I8">
+        <v>300</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="0"/>
         <v>5.17240234375</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>15</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>5296.54</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M8">
+        <v>1.8919999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>50</v>
       </c>
@@ -3428,17 +3631,23 @@
         <v>29.799635410308841</v>
       </c>
       <c r="I9">
+        <v>310</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="0"/>
         <v>5.2354003906250002</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>15</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>5361.05</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M9">
+        <v>1.9370000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>50</v>
       </c>
@@ -3464,17 +3673,23 @@
         <v>10.4386875629425</v>
       </c>
       <c r="I10">
+        <v>290</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="0"/>
         <v>5.0866894531250004</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>14</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>5208.7700000000004</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M10">
+        <v>1.387</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>50</v>
       </c>
@@ -3500,17 +3715,23 @@
         <v>167.4226031303406</v>
       </c>
       <c r="I11">
+        <v>337</v>
+      </c>
+      <c r="J11">
         <f t="shared" si="0"/>
         <v>5.4858496093750002</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>16</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>5617.51</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M11">
+        <v>9.7720000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>100</v>
       </c>
@@ -3536,17 +3757,23 @@
         <v>63.744473218917847</v>
       </c>
       <c r="I12">
+        <v>576</v>
+      </c>
+      <c r="J12">
         <f t="shared" si="0"/>
         <v>9.9217675781249994</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>28</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>10159.89</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M12">
+        <v>9.1270000000000007</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>100</v>
       </c>
@@ -3572,17 +3799,23 @@
         <v>73.317306280136108</v>
       </c>
       <c r="I13">
+        <v>580</v>
+      </c>
+      <c r="J13">
         <f t="shared" si="0"/>
         <v>10.203974609375001</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>28</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>10448.870000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M13">
+        <v>3.9580000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>100</v>
       </c>
@@ -3608,17 +3841,23 @@
         <v>80.461363554000854</v>
       </c>
       <c r="I14">
+        <v>607</v>
+      </c>
+      <c r="J14">
         <f t="shared" si="0"/>
         <v>10.282753906250001</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>28</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>10529.54</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M14">
+        <v>4.327</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>100</v>
       </c>
@@ -3644,17 +3883,23 @@
         <v>17.870550155639648</v>
       </c>
       <c r="I15">
+        <v>555</v>
+      </c>
+      <c r="J15">
         <f t="shared" si="0"/>
         <v>10.002744140625</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>26</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>10242.81</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M15">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>100</v>
       </c>
@@ -3680,14 +3925,20 @@
         <v>651.26701760292053</v>
       </c>
       <c r="I16">
+        <v>710</v>
+      </c>
+      <c r="J16">
         <f t="shared" si="0"/>
         <v>11.391787109375</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>30</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>11665.19</v>
+      </c>
+      <c r="M16">
+        <v>20.524000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3696,9 +3947,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85EFFC09-E175-46E6-84C2-1C8534DC4F16}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -3707,10 +3958,12 @@
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -3733,19 +3986,25 @@
         <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M1" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>25</v>
       </c>
@@ -3771,17 +4030,23 @@
         <v>40.761738777160637</v>
       </c>
       <c r="I2">
-        <f>K2/1024</f>
+        <v>310</v>
+      </c>
+      <c r="J2">
+        <f>L2/1024</f>
         <v>4.6024023437499997</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>8.9</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>4712.8599999999997</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>3.9950000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>25</v>
       </c>
@@ -3807,17 +4072,23 @@
         <v>24.485044002532959</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I16" si="0">K3/1024</f>
+        <v>312</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J16" si="0">L3/1024</f>
         <v>4.8210546875000002</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>8.9</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>4936.76</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M3">
+        <v>6.1680000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>25</v>
       </c>
@@ -3843,17 +4114,23 @@
         <v>26.01601600646973</v>
       </c>
       <c r="I4">
+        <v>335</v>
+      </c>
+      <c r="J4">
         <f t="shared" si="0"/>
         <v>4.8794628906249997</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>8.9</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>4996.57</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M4">
+        <v>6.149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>25</v>
       </c>
@@ -3879,17 +4156,23 @@
         <v>11.070473194122309</v>
       </c>
       <c r="I5">
+        <v>299</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="0"/>
         <v>4.6653124999999998</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>8.5</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>4777.28</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M5">
+        <v>5.6890000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>25</v>
       </c>
@@ -3915,17 +4198,23 @@
         <v>69.02873969078064</v>
       </c>
       <c r="I6">
+        <v>350</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="0"/>
         <v>8.3837695312499996</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>10</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>8584.98</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M6">
+        <v>15.554</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>50</v>
       </c>
@@ -3951,17 +4240,23 @@
         <v>68.332580327987671</v>
       </c>
       <c r="I7">
+        <v>572</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="0"/>
         <v>9.3940136718749994</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>20</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>9619.4699999999993</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M7">
+        <v>6.2949999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>50</v>
       </c>
@@ -3987,17 +4282,23 @@
         <v>42.846899271011353</v>
       </c>
       <c r="I8">
+        <v>575</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="0"/>
         <v>9.7616992187499996</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>20</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>9995.98</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M8">
+        <v>9.8119999999999994</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>50</v>
       </c>
@@ -4023,17 +4324,23 @@
         <v>44.150554180145257</v>
       </c>
       <c r="I9">
+        <v>612</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="0"/>
         <v>9.9270214843750004</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>20</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>10165.27</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M9">
+        <v>9.9960000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>50</v>
       </c>
@@ -4059,17 +4366,23 @@
         <v>19.841279983520511</v>
       </c>
       <c r="I10">
+        <v>558</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="0"/>
         <v>9.5826562499999994</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>18</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>9812.64</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M10">
+        <v>8.9749999999999996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>50</v>
       </c>
@@ -4095,17 +4408,23 @@
         <v>107.7042288780212</v>
       </c>
       <c r="I11">
+        <v>594</v>
+      </c>
+      <c r="J11">
         <f t="shared" si="0"/>
         <v>16.019482421875001</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>25</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>16403.95</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M11">
+        <v>37.07</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>100</v>
       </c>
@@ -4131,17 +4450,23 @@
         <v>103.0709517002106</v>
       </c>
       <c r="I12">
+        <v>574</v>
+      </c>
+      <c r="J12">
         <f t="shared" si="0"/>
         <v>10.142177734375</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>28</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>10385.59</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M12">
+        <v>10.163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>100</v>
       </c>
@@ -4167,17 +4492,23 @@
         <v>51.531718015670783</v>
       </c>
       <c r="I13">
+        <v>577</v>
+      </c>
+      <c r="J13">
         <f t="shared" si="0"/>
         <v>10.400078125</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>28</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>10649.68</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M13">
+        <v>15.339</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>100</v>
       </c>
@@ -4203,17 +4534,23 @@
         <v>55.438335657119751</v>
       </c>
       <c r="I14">
+        <v>615</v>
+      </c>
+      <c r="J14">
         <f t="shared" si="0"/>
         <v>10.556064453125</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>28</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>10809.41</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M14">
+        <v>15.397</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>100</v>
       </c>
@@ -4239,17 +4576,23 @@
         <v>19.46701288223267</v>
       </c>
       <c r="I15">
+        <v>559</v>
+      </c>
+      <c r="J15">
         <f t="shared" si="0"/>
         <v>10.21271484375</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>27</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>10457.82</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M15">
+        <v>14.45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>100</v>
       </c>
@@ -4275,14 +4618,20 @@
         <v>126.7946817874908</v>
       </c>
       <c r="I16">
+        <v>644</v>
+      </c>
+      <c r="J16">
         <f t="shared" si="0"/>
         <v>21.79001953125</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>35</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>22312.98</v>
+      </c>
+      <c r="M16">
+        <v>83.488</v>
       </c>
     </row>
   </sheetData>
@@ -4290,9 +4639,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8F966A1-A5E4-4208-BD66-2FCB92AA77B6}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -4301,9 +4650,12 @@
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -4326,19 +4678,25 @@
         <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M1" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>25</v>
       </c>
@@ -4364,17 +4722,23 @@
         <v>4.1363911628723136</v>
       </c>
       <c r="I2">
-        <f>K2/1024</f>
+        <v>145</v>
+      </c>
+      <c r="J2">
+        <f>L2/1024</f>
         <v>2.3379589843750002</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>6.9</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>2394.0700000000002</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>0.20300000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>25</v>
       </c>
@@ -4400,17 +4764,23 @@
         <v>11.170616388320919</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I16" si="0">K3/1024</f>
+        <v>151</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J16" si="0">L3/1024</f>
         <v>3.0250878906250001</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>6.9</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>3097.69</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M3">
+        <v>0.64500000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>25</v>
       </c>
@@ -4436,17 +4806,23 @@
         <v>12.288981676101679</v>
       </c>
       <c r="I4">
+        <v>153</v>
+      </c>
+      <c r="J4">
         <f t="shared" si="0"/>
         <v>3.0593945312500002</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>6.9</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>3132.82</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M4">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>25</v>
       </c>
@@ -4472,17 +4848,23 @@
         <v>5.1880824565887451</v>
       </c>
       <c r="I5">
+        <v>145</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="0"/>
         <v>2.9044531249999999</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>6.8</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>2974.16</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M5">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>25</v>
       </c>
@@ -4508,17 +4890,23 @@
         <v>18.046691417694088</v>
       </c>
       <c r="I6">
+        <v>156</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="0"/>
         <v>3.22408203125</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>7</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>3301.46</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M6">
+        <v>1.2430000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>50</v>
       </c>
@@ -4544,17 +4932,23 @@
         <v>5.659299373626709</v>
       </c>
       <c r="I7">
+        <v>281</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="0"/>
         <v>4.5110742187500001</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>18</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>4619.34</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M7">
+        <v>0.20200000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>50</v>
       </c>
@@ -4580,17 +4974,23 @@
         <v>18.77040600776672</v>
       </c>
       <c r="I8">
+        <v>294</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="0"/>
         <v>5.9237792968749998</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>18</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>6065.95</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M8">
+        <v>1.2230000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>50</v>
       </c>
@@ -4616,17 +5016,23 @@
         <v>21.01609110832214</v>
       </c>
       <c r="I9">
+        <v>295</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="0"/>
         <v>6.0237695312500001</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>18.5</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>6168.34</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M9">
+        <v>1.3140000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>50</v>
       </c>
@@ -4652,17 +5058,23 @@
         <v>10.25874972343445</v>
       </c>
       <c r="I10">
+        <v>284</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="0"/>
         <v>5.7982031249999997</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>18</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>5937.36</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M10">
+        <v>0.56699999999999995</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>50</v>
       </c>
@@ -4688,17 +5100,23 @@
         <v>31.889566421508789</v>
       </c>
       <c r="I11">
+        <v>298</v>
+      </c>
+      <c r="J11">
         <f t="shared" si="0"/>
         <v>6.2085546875000004</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>25</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>6357.56</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M11">
+        <v>5.5019999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>100</v>
       </c>
@@ -4724,17 +5142,23 @@
         <v>11.382223129272459</v>
       </c>
       <c r="I12">
+        <v>553</v>
+      </c>
+      <c r="J12">
         <f t="shared" si="0"/>
         <v>8.7917871093750009</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>28</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>9002.7900000000009</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M12">
+        <v>0.21299999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>100</v>
       </c>
@@ -4760,17 +5184,23 @@
         <v>78.243307590484619</v>
       </c>
       <c r="I13">
+        <v>587</v>
+      </c>
+      <c r="J13">
         <f t="shared" si="0"/>
         <v>11.212705078125</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>28</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>11481.81</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M13">
+        <v>3.6469999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>100</v>
       </c>
@@ -4796,17 +5226,23 @@
         <v>80.169402360916138</v>
       </c>
       <c r="I14">
+        <v>591</v>
+      </c>
+      <c r="J14">
         <f t="shared" si="0"/>
         <v>11.276064453125</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>28</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>11546.69</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M14">
+        <v>3.8439999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>100</v>
       </c>
@@ -4832,17 +5268,23 @@
         <v>16.579630851745609</v>
       </c>
       <c r="I15">
+        <v>556</v>
+      </c>
+      <c r="J15">
         <f t="shared" si="0"/>
         <v>10.96337890625</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>28</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>11226.5</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M15">
+        <v>1.2589999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>100</v>
       </c>
@@ -4868,14 +5310,20 @@
         <v>101.16583561897281</v>
       </c>
       <c r="I16">
+        <v>600</v>
+      </c>
+      <c r="J16">
         <f t="shared" si="0"/>
         <v>11.588759765624999</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>35</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>11866.89</v>
+      </c>
+      <c r="M16">
+        <v>13.117000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -4884,7 +5332,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35DA226-F5A6-4A98-8238-6D1555C1E612}">
   <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4896,6 +5344,7 @@
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -4953,15 +5402,18 @@
         <v>94.283569999999997</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>0.60499999999999998</v>
       </c>
       <c r="H2">
-        <v>5.9769800000000002</v>
+        <v>30.976980000000001</v>
       </c>
       <c r="I2">
         <f>K2/1024</f>
         <v>1.27201171875</v>
       </c>
+      <c r="J2">
+        <v>6.8</v>
+      </c>
       <c r="K2">
         <v>1302.54</v>
       </c>
@@ -4986,15 +5438,18 @@
         <v>92.511350100000001</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>0.70099999999999996</v>
       </c>
       <c r="H3">
-        <v>25.300184249800001</v>
+        <v>144.3001842498</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I7" si="0">K3/1024</f>
         <v>1.2906445312499999</v>
       </c>
+      <c r="J3">
+        <v>13.7</v>
+      </c>
       <c r="K3">
         <v>1321.62</v>
       </c>
@@ -5019,15 +5474,18 @@
         <v>107.88930000000001</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>0.746</v>
       </c>
       <c r="H4">
-        <v>34.277099999999997</v>
+        <v>228.27709999999999</v>
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
         <v>1.3832421875000001</v>
       </c>
+      <c r="J4">
+        <v>40.799999999999997</v>
+      </c>
       <c r="K4">
         <v>1416.44</v>
       </c>
@@ -5049,18 +5507,21 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>34.06756</v>
+        <v>214.06755999999999</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="H5">
-        <v>34.06756</v>
+        <v>204.06755999999999</v>
       </c>
       <c r="I5">
         <f t="shared" si="0"/>
         <v>1.633994140625</v>
       </c>
+      <c r="J5">
+        <v>15</v>
+      </c>
       <c r="K5">
         <v>1673.21</v>
       </c>
@@ -5082,18 +5543,21 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>60.285357585</v>
+        <v>400.28535758499999</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>0.745</v>
       </c>
       <c r="H6">
-        <v>60.285357585</v>
+        <v>360.28535758499999</v>
       </c>
       <c r="I6">
         <f t="shared" si="0"/>
         <v>1.844951171875</v>
       </c>
+      <c r="J6">
+        <v>39</v>
+      </c>
       <c r="K6">
         <v>1889.23</v>
       </c>
@@ -5115,18 +5579,21 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>76.277760000000001</v>
+        <v>468.27776</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>0.76100000000000001</v>
       </c>
       <c r="H7">
-        <v>76.277760000000001</v>
+        <v>456.27776</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
         <v>2.008994140625</v>
       </c>
+      <c r="J7">
+        <v>49.2</v>
+      </c>
       <c r="K7">
         <v>2057.21</v>
       </c>
@@ -5134,91 +5601,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D448E8-895B-453C-BC61-2624AF8420AB}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2">
-        <v>6.3574999999999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3">
-        <v>94.953100000000006</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4">
-        <v>29.642399999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B5">
-        <v>3.3828</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6">
-        <v>1.6611</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7">
-        <v>43.620800000000003</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8">
-        <v>0.41070000000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9">
-        <v>0.52849999999999997</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>